<commit_message>
work on career & enquiry form
</commit_message>
<xml_diff>
--- a/backend/enquiry.xlsx
+++ b/backend/enquiry.xlsx
@@ -427,28 +427,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Ismat</v>
+        <v>ismat</v>
       </c>
       <c r="B2" t="str">
-        <v>8888888888</v>
+        <v>9999999999</v>
       </c>
       <c r="C2" t="str">
         <v>ismat@gmail.com</v>
       </c>
       <c r="D2" t="str">
-        <v>zylow</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>Web App</v>
+        <v>Website</v>
       </c>
       <c r="F2" t="str">
-        <v>1 Month</v>
+        <v>Later</v>
       </c>
       <c r="G2" t="str">
-        <v>efghi</v>
+        <v>abc</v>
       </c>
       <c r="H2" t="str">
-        <v>5/1/2026, 2:29:52 PM</v>
+        <v>6/12/2026, 11:04:13 AM</v>
       </c>
     </row>
   </sheetData>

</xml_diff>